<commit_message>
Finalização do modelo do grafico
</commit_message>
<xml_diff>
--- a/Novo(a) Planilha do Microsoft Excel.xlsx
+++ b/Novo(a) Planilha do Microsoft Excel.xlsx
@@ -1,29 +1,76 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heitor.dias\Desktop\Projeto-RPG\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9D403D-D5B2-4159-AE33-CC6A9ABA7100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
+  <si>
+    <t>button -&gt;</t>
+  </si>
+  <si>
+    <t>&lt;- button</t>
+  </si>
+  <si>
+    <t>clear</t>
+  </si>
+  <si>
+    <t>Overheat</t>
+  </si>
+  <si>
+    <t>Cold</t>
+  </si>
+  <si>
+    <t>Invisivel</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -49,8 +96,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -66,6 +123,892 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Heat</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="9.9328220956013916E-2"/>
+          <c:y val="0.18316049382716051"/>
+          <c:w val="0.80134403779308783"/>
+          <c:h val="0.64955497229512982"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Heat</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-525E-4DC9-B988-EC6B22182C07}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-525E-4DC9-B988-EC6B22182C07}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000006-525E-4DC9-B988-EC6B22182C07}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>(Plan1!$B$13,Plan1!$D$13,Plan1!$C$13)</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Overheat</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cold</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Invisivel</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>(Plan1!$B$15,Plan1!$D$15,Plan1!$D$12)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-525E-4DC9-B988-EC6B22182C07}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="270"/>
+        <c:holeSize val="65"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="11">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent5"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>43603</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>173671</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>571560</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>146456</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Gráfico 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B932B7D-96A6-FA0F-10F5-3DC08CB0E94E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +1273,108 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B12:X15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <f>SUM(C14,D15)</f>
+        <v>8</v>
+      </c>
+      <c r="M12">
+        <f>SUM(L14,M15)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>8</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L14" s="1">
+        <v>5</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="V14" s="1"/>
+      <c r="W14" s="1"/>
+      <c r="X14" s="1"/>
+    </row>
+    <row r="15" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B15" s="4">
+        <f>C14</f>
+        <v>8</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4">
+        <f>8-C14</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="4">
+        <f>L14</f>
+        <v>5</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M15" s="4">
+        <f>12-L14</f>
+        <v>7</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="3"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="3"/>
+      <c r="V15" s="2"/>
+      <c r="W15" s="1"/>
+      <c r="X15" s="3"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
finalização do grafico de combustivel e atualização de design
</commit_message>
<xml_diff>
--- a/Novo(a) Planilha do Microsoft Excel.xlsx
+++ b/Novo(a) Planilha do Microsoft Excel.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heitor.dias\Desktop\Projeto-RPG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9D403D-D5B2-4159-AE33-CC6A9ABA7100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86492C0-2F42-4ABF-A8D4-45C11D4F2EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15945" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dados" sheetId="1" r:id="rId1"/>
+    <sheet name="Console" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
   <si>
     <t>button -&gt;</t>
   </si>
@@ -54,6 +55,12 @@
   </si>
   <si>
     <t>Invisivel</t>
+  </si>
+  <si>
+    <t>Gasolina (l)</t>
+  </si>
+  <si>
+    <t>Capacidade total (l)</t>
   </si>
 </sst>
 </file>
@@ -96,16 +103,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -160,7 +164,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Heat</a:t>
+              <a:t>Heat (8x)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -274,7 +278,7 @@
           </c:dPt>
           <c:cat>
             <c:strRef>
-              <c:f>(Plan1!$B$13,Plan1!$D$13,Plan1!$C$13)</c:f>
+              <c:f>(Dados!$B$13,Dados!$D$13,Dados!$C$13)</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -291,15 +295,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>(Plan1!$B$15,Plan1!$D$15,Plan1!$D$12)</c:f>
+              <c:f>(Dados!$B$15,Dados!$D$15,Dados!$D$12)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>8</c:v>
@@ -310,6 +314,1217 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-525E-4DC9-B988-EC6B22182C07}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="270"/>
+        <c:holeSize val="65"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Heat (12x)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="9.9328220956013916E-2"/>
+          <c:y val="0.18316049382716051"/>
+          <c:w val="0.80134403779308783"/>
+          <c:h val="0.64955497229512982"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Heat</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-210B-4513-9FA3-76706507710A}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-210B-4513-9FA3-76706507710A}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-210B-4513-9FA3-76706507710A}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>(Dados!$B$13,Dados!$D$13,Dados!$C$13)</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Overheat</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cold</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Invisivel</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>(Dados!$F$15,Dados!$H$15,Dados!$H$12)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-210B-4513-9FA3-76706507710A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="270"/>
+        <c:holeSize val="65"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1000" baseline="0"/>
+              <a:t>Gasolina (litros)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dados!$J$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Gasolina (l)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Gasosa total</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dados!$J$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9413-47A4-A12B-3FCEE962DD7B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Capacidade maxima</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-9413-47A4-A12B-3FCEE962DD7B}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:val>
+            <c:numRef>
+              <c:f>Dados!$K$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-9413-47A4-A12B-3FCEE962DD7B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="451202464"/>
+        <c:axId val="451202944"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="451202464"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="451202944"/>
+        <c:crossesAt val="0"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="451202944"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="451202464"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Heat (8)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="9.9328220956013916E-2"/>
+          <c:y val="0.18316049382716051"/>
+          <c:w val="0.80134403779308783"/>
+          <c:h val="0.64955497229512982"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Heat</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-C2F8-49B1-8224-78903E25B131}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-C2F8-49B1-8224-78903E25B131}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="19050">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-C2F8-49B1-8224-78903E25B131}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>(Dados!$B$13,Dados!$D$13,Dados!$C$13)</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Overheat</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cold</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Invisivel</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>(Dados!$B$15,Dados!$D$15,Dados!$D$12)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-C2F8-49B1-8224-78903E25B131}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="270"/>
+        <c:holeSize val="65"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Heat (12)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="9.9328220956013916E-2"/>
+          <c:y val="0.18316049382716051"/>
+          <c:w val="0.80134403779308783"/>
+          <c:h val="0.64955497229512982"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Heat</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-41EC-4CA7-84EE-0EA4FB5B904A}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-41EC-4CA7-84EE-0EA4FB5B904A}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-41EC-4CA7-84EE-0EA4FB5B904A}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>(Dados!$B$13,Dados!$D$13,Dados!$C$13)</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Overheat</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cold</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Invisivel</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>(Dados!$F$15,Dados!$H$15,Dados!$H$12)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-41EC-4CA7-84EE-0EA4FB5B904A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -449,7 +1664,2218 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="11">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent5"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="11">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent5"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="11">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent5"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -1003,6 +4429,161 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>11906</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>154781</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>539863</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>127566</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Gráfico 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A468F923-000E-428D-93ED-67FED93124BE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>322385</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>359019</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>161192</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Gráfico 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27B77094-0A5F-2902-696F-DF04EF416EF6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>513669</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>153760</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Gráfico 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{186B1F41-6CEA-4AC3-B6F4-8AD76C51893D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>608919</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>144235</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Gráfico 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAB60720-D4F3-4B0C-BAC9-73BDB209A01D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1274,16 +4855,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Planilha1"/>
   <dimension ref="B12:X15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="12" spans="2:24" x14ac:dyDescent="0.25">
       <c r="D12">
         <f>SUM(C14,D15)</f>
         <v>8</v>
       </c>
-      <c r="M12">
-        <f>SUM(L14,M15)</f>
+      <c r="H12">
+        <f>SUM(G14,H15)</f>
         <v>12</v>
       </c>
     </row>
@@ -1297,14 +4883,20 @@
       <c r="D13" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="2:24" x14ac:dyDescent="0.25">
@@ -1312,21 +4904,25 @@
         <v>1</v>
       </c>
       <c r="C14" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L14" s="1">
-        <v>5</v>
+      <c r="G14" s="1">
+        <v>7</v>
       </c>
-      <c r="M14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>0</v>
+      </c>
+      <c r="J14" s="1">
+        <v>12</v>
+      </c>
+      <c r="K14" s="1">
+        <v>25</v>
       </c>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
@@ -1339,30 +4935,29 @@
       <c r="X14" s="1"/>
     </row>
     <row r="15" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B15" s="4">
+      <c r="B15" s="1">
         <f>C14</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="1">
         <f>8-C14</f>
-        <v>0</v>
+        <v>3</v>
       </c>
-      <c r="F15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="4">
-        <f>L14</f>
+      <c r="F15" s="1">
+        <f>G14</f>
+        <v>7</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H15" s="1">
+        <f>12-G14</f>
         <v>5</v>
       </c>
-      <c r="L15" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="M15" s="4">
-        <f>12-L14</f>
-        <v>7</v>
-      </c>
+      <c r="J15" s="2"/>
       <c r="N15" s="2"/>
       <c r="O15" s="1"/>
       <c r="P15" s="3"/>
@@ -1377,4 +4972,15 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{335E0B7F-650C-46F2-AC3E-832E737E5316}">
+  <sheetPr codeName="Planilha2"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>